<commit_message>
Mise a jour du 06-09-2026 23:05:31,37
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="1" state="visible" r:id="rId1"/>
@@ -401,25 +401,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U178"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.26953125" defaultRowHeight="14.5"/>
+  <dimension ref="A1:U187"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="2.90625" customWidth="1" style="1" min="1" max="1"/>
-    <col width="4.6328125" customWidth="1" style="1" min="2" max="2"/>
-    <col width="4.453125" customWidth="1" style="1" min="3" max="3"/>
-    <col width="3.1796875" customWidth="1" style="1" min="4" max="4"/>
-    <col width="44.08984375" customWidth="1" style="1" min="5" max="5"/>
-    <col width="3.26953125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="2.921875" customWidth="1" style="1" min="1" max="1"/>
+    <col width="4.61328125" customWidth="1" style="1" min="2" max="2"/>
+    <col width="4.4609375" customWidth="1" style="1" min="3" max="3"/>
+    <col width="3.15234375" customWidth="1" style="1" min="4" max="4"/>
+    <col width="44.07421875" customWidth="1" style="1" min="5" max="5"/>
+    <col width="3.23046875" customWidth="1" style="1" min="7" max="7"/>
     <col width="7" customWidth="1" style="1" min="8" max="8"/>
-    <col width="2.26953125" customWidth="1" style="1" min="10" max="10"/>
-    <col width="3.90625" customWidth="1" style="1" min="11" max="11"/>
-    <col width="1.90625" customWidth="1" style="1" min="13" max="13"/>
-    <col width="2.7265625" customWidth="1" style="1" min="14" max="14"/>
-    <col width="2.36328125" customWidth="1" style="1" min="16" max="16"/>
-    <col width="2.26953125" customWidth="1" style="1" min="17" max="17"/>
+    <col width="2.23046875" customWidth="1" style="1" min="10" max="10"/>
+    <col width="3.921875" customWidth="1" style="1" min="11" max="11"/>
+    <col width="1.921875" customWidth="1" style="1" min="13" max="13"/>
+    <col width="2.69140625" customWidth="1" style="1" min="14" max="14"/>
+    <col width="2.3828125" customWidth="1" style="1" min="16" max="16"/>
+    <col width="2.23046875" customWidth="1" style="1" min="17" max="17"/>
     <col width="2" customWidth="1" style="1" min="19" max="19"/>
-    <col width="2.26953125" customWidth="1" style="1" min="20" max="20"/>
-    <col width="18.26953125" customWidth="1" style="1" min="21" max="21"/>
+    <col width="2.23046875" customWidth="1" style="1" min="20" max="20"/>
+    <col width="18.23046875" customWidth="1" style="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -854,351 +854,219 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
         <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>T.SF2.1</t>
+          <t>T.SF0.1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Vecteur</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11" ht="29.15" customHeight="1" s="1">
+          <t>Utiliser le symbole Somme</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>pBAOi2-dJ30</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>208</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>_kqhfSz8DWY</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="10" s="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>T.SF0.2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Utiliser une boucle Pour (for)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>o8AEP07TIMw</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>226</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>9lOP2H54twE</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>491</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Juste regarder</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" s="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
         <v>3</v>
       </c>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>T.SF3.1</t>
+          <t>T.SF0.3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>0NBWe0RRjG4</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>591</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>BKt3SwTxykI</t>
+          <t>Calculer une somme (for)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>jjOwu42rsDg</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>77</v>
+      </c>
+      <c r="H11" t="n">
+        <v>249</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>DGz8PCl-B_8</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="12" ht="29.15" customHeight="1" s="1">
+        <v>471</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Juste regarder</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" s="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>T.SF3.2</t>
+          <t>T.SF0.4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Additionner des limites</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>CEAbo1PoGl8</t>
+          <t>Faire une Liste (for)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>97hQwXafiuM</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="13" ht="29.15" customHeight="1" s="1">
+        <v>350</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Juste regarder</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>T.SF3.3</t>
+          <t>T.SF0.5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Produit et Quotient de limite</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>FU5_5FDsoSw</t>
+          <t xml:space="preserve">Coder un seuil </t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>5M8cMnHj2Xk</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>561</v>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>OkpadGbc5zc</t>
+        <v>357</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>vJmpzwhaka8</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="14" ht="29.15" customHeight="1" s="1">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>T.SF3.4</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Lever une indétermination en factorisant</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Gh8KXArr1hk</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>760</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>7rz7td0LZGY</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>223</v>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>jCFejEo2oQY</t>
-        </is>
-      </c>
-      <c r="N14" t="n">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="15" ht="29.15" customHeight="1" s="1">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" t="n">
-        <v>5</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>T.SF3.5</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Lever une indétermination avec des racines carrés</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="L15" s="3" t="inlineStr">
-        <is>
-          <t>JbDvz3iobMk</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>275</v>
-      </c>
-      <c r="O15" s="3" t="n"/>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>HNxF6K5mvvk</t>
-        </is>
-      </c>
-      <c r="T15" t="n">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C16" t="n">
-        <v>6</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>T.SF3.6</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Utiliser le théorème de comparaison</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" t="n">
-        <v>7</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>T.SF3.7</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C18" t="n">
-        <v>8</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>T.SF3.8</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Justifier la convergence d'une suite</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="29.15" customHeight="1" s="1">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
-      </c>
-      <c r="C19" t="n">
-        <v>9</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>T.SF3.9</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Limite d'une suite géométrique</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>oE7SS7T9PBM</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>434</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>MEp55lywR0M</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>274</v>
-      </c>
-      <c r="L19" s="3" t="inlineStr">
-        <is>
-          <t>HAcgnHFkVCc</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>470</v>
-      </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>kMelIoA4E2o</t>
-        </is>
-      </c>
-      <c r="Q19" t="n">
-        <v>764</v>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Méthode 1p51</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
+        <v>325</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>GngW7W1FEBU</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="14" s="1"/>
+    <row r="15" s="1"/>
+    <row r="16" s="1"/>
+    <row r="17" s="1"/>
+    <row r="18" s="1"/>
+    <row r="19" s="1"/>
+    <row r="20" ht="29.15" customHeight="1" s="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>T</t>
@@ -1207,8 +1075,37 @@
       <c r="B20" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" ht="43.75" customHeight="1" s="1">
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>T.SF3.1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>0NBWe0RRjG4</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>591</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>BKt3SwTxykI</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="21" ht="29.15" customHeight="1" s="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>T</t>
@@ -1218,28 +1115,28 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>T.SF3.8</t>
+          <t>T.SF3.2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>a recaser</t>
+          <t>Additionner des limites</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>ns-Hq9uVbS0</t>
+          <t>CEAbo1PoGl8</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="22" ht="29.15" customHeight="1" s="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>T</t>
@@ -1248,19 +1145,123 @@
       <c r="B22" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="23">
+      <c r="C22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>T.SF3.3</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Produit et Quotient de limite</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>FU5_5FDsoSw</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>561</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>OkpadGbc5zc</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="23" ht="29.15" customHeight="1" s="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-    </row>
-    <row r="24">
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>T.SF3.4</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Lever une indétermination en factorisant</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Gh8KXArr1hk</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>760</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>7rz7td0LZGY</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>223</v>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>jCFejEo2oQY</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" ht="29.15" customHeight="1" s="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>T</t>
         </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>T.SF3.5</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Lever une indétermination avec des racines carrés</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>JbDvz3iobMk</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>275</v>
+      </c>
+      <c r="O24" s="3" t="n"/>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>HNxF6K5mvvk</t>
+        </is>
+      </c>
+      <c r="T24" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="25">
@@ -1269,6 +1270,22 @@
           <t>T</t>
         </is>
       </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>T.SF3.6</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème de comparaison</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1276,6 +1293,22 @@
           <t>T</t>
         </is>
       </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>T.SF3.7</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1283,11 +1316,80 @@
           <t>T</t>
         </is>
       </c>
-    </row>
-    <row r="28">
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Justifier la convergence d'une suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="29.15" customHeight="1" s="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>T</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>T.SF3.9</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Limite d'une suite géométrique</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>oE7SS7T9PBM</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>434</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>MEp55lywR0M</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>274</v>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>HAcgnHFkVCc</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>470</v>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>kMelIoA4E2o</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>764</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Méthode 1p51</t>
         </is>
       </c>
     </row>
@@ -1297,12 +1399,39 @@
           <t>T</t>
         </is>
       </c>
-    </row>
-    <row r="30">
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" ht="43.75" customHeight="1" s="1">
       <c r="A30" t="inlineStr">
         <is>
           <t>T</t>
         </is>
+      </c>
+      <c r="B30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" t="n">
+        <v>8</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>a recaser</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>ns-Hq9uVbS0</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>567</v>
       </c>
     </row>
     <row r="31">
@@ -1311,6 +1440,9 @@
           <t>T</t>
         </is>
       </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2336,6 +2468,69 @@
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
         <is>
           <t>T</t>
         </is>
@@ -2353,13 +2548,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.08984375" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="11.08984375" customWidth="1" style="1" min="1" max="1"/>
+    <col width="11.07421875" customWidth="1" style="1" min="1" max="1"/>
     <col width="60" customWidth="1" style="1" min="2" max="2"/>
-    <col width="2.7265625" customWidth="1" style="1" min="3" max="237"/>
-    <col width="11.08984375" customWidth="1" style="1" min="238" max="238"/>
-    <col width="11.08984375" customWidth="1" style="1" min="239" max="16384"/>
+    <col width="2.69140625" customWidth="1" style="1" min="3" max="237"/>
+    <col width="11.07421875" customWidth="1" style="1" min="238" max="239"/>
+    <col width="11.07421875" customWidth="1" style="1" min="240" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="59.15" customHeight="1" s="1">
@@ -3203,28 +3398,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T.SF2.1</t>
+          <t>T.SF0.1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vecteur</t>
+          <t>Utiliser le symbole Somme</t>
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T.SF0.2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Utiliser une boucle Pour (for)</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>T.SF3.1</t>
+          <t>T.SF0.3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
+          <t>Calculer une somme (for)</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -3232,12 +3437,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>T.SF3.2</t>
+          <t>T.SF0.4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Additionner des limites</t>
+          <t>Faire une Liste (for)</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
@@ -3245,135 +3450,165 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>T.SF3.3</t>
+          <t>T.SF0.5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Produit et Quotient de limite</t>
+          <t xml:space="preserve">Coder un seuil </t>
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>T.SF3.4</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Lever une indétermination en factorisant</t>
-        </is>
-      </c>
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>T.SF3.5</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Lever une indétermination avec des racines carrés</t>
-        </is>
-      </c>
       <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>T.SF3.6</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Utiliser le théorème de comparaison</t>
-        </is>
-      </c>
       <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>T.SF3.7</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
-        </is>
-      </c>
       <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>T.SF3.8</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Justifier la convergence d'une suite</t>
-        </is>
-      </c>
       <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>T.SF3.9</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Limite d'une suite géométrique</t>
-        </is>
-      </c>
       <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>T.SF3.1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
+        </is>
+      </c>
       <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>T.SF3.2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Additionner des limites</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T.SF3.3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Produit et Quotient de limite</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T.SF3.4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Lever une indétermination en factorisant</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>T.SF3.5</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lever une indétermination avec des racines carrés</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>T.SF3.6</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème de comparaison</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>T.SF3.7</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>T.SF3.8</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>a recaser</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="n"/>
-    </row>
-    <row r="22">
-      <c r="H22" s="2" t="n"/>
-    </row>
-    <row r="23">
-      <c r="H23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="H24" s="2" t="n"/>
-    </row>
-    <row r="25">
-      <c r="H25" s="2" t="n"/>
-    </row>
-    <row r="26">
-      <c r="H26" s="2" t="n"/>
-    </row>
-    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Justifier la convergence d'une suite</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>T.SF3.9</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Limite d'une suite géométrique</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>a recaser</t>
+        </is>
+      </c>
       <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
@@ -3988,9 +4223,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <cols>
-    <col width="3.7265625" customWidth="1" style="1" min="2" max="43"/>
+    <col width="3.69140625" customWidth="1" style="1" min="2" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4269,7 +4504,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Mise a jour du 07-09-2026 15:56:06.21
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFDAF280-8D9C-4EB1-8901-3DEF3E023EB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03BFA44-C500-4385-A349-B7F8F1CAB020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="133">
   <si>
     <t>Préfixe</t>
   </si>
@@ -3035,9 +3035,7 @@
       <c r="X2" t="s">
         <v>113</v>
       </c>
-      <c r="Z2" t="s">
-        <v>113</v>
-      </c>
+      <c r="Z2"/>
     </row>
     <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -3062,6 +3060,9 @@
       <c r="Y4" t="s">
         <v>113</v>
       </c>
+      <c r="AA4" s="1" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -3071,9 +3072,10 @@
         <v>39</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="Z5" t="s">
+      <c r="Y5" s="1" t="s">
         <v>113</v>
       </c>
+      <c r="Z5"/>
     </row>
     <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -3083,6 +3085,9 @@
         <v>45</v>
       </c>
       <c r="H6" s="2"/>
+      <c r="Z6" s="1" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A7" t="s">

</xml_diff>

<commit_message>
Mise a jour du 07-09-2026 17:51:53.80
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03BFA44-C500-4385-A349-B7F8F1CAB020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F072AF-2D91-4340-9A48-C1F0E30B3DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="133">
   <si>
     <t>Préfixe</t>
   </si>
@@ -3032,9 +3032,7 @@
       <c r="V2" t="s">
         <v>113</v>
       </c>
-      <c r="X2" t="s">
-        <v>113</v>
-      </c>
+      <c r="X2"/>
       <c r="Z2"/>
     </row>
     <row r="3" spans="1:237" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Mise a jour du 21-09-2026 11:16:11.32
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC59BA7-655D-446D-8CD9-1916E09502EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB04A768-B21E-49B1-A0AA-FD1CD1CB5651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="14370" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -18,19 +18,8 @@
     <sheet name="Calendrier" sheetId="3" r:id="rId3"/>
     <sheet name="liste date semaine" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -308,15 +297,18 @@
     <t>KP3E-p5zbVo</t>
   </si>
   <si>
+    <t>DA54wBn78fQ</t>
+  </si>
+  <si>
+    <t>T.SF2.4</t>
+  </si>
+  <si>
+    <t>Savoir démontrer que des points sont coplanaires (sans coord)</t>
+  </si>
+  <si>
     <t>i4jDkJNtzZg</t>
   </si>
   <si>
-    <t>T.SF2.4</t>
-  </si>
-  <si>
-    <t>Savoir démontrer que des points sont coplanaires (sans coord)</t>
-  </si>
-  <si>
     <t>T.SF2.5</t>
   </si>
   <si>
@@ -551,10 +543,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>DA54wBn78fQ</t>
-  </si>
-  <si>
-    <t>v=_ev35SGD_tE</t>
+    <t>_ev35SGD_tE</t>
   </si>
 </sst>
 </file>
@@ -881,27 +870,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U190"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.84375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.69140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.07421875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.23046875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="3.921875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.23046875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.84375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.84375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="3.921875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="2.4609375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.53515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="3.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="3.88671875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="2.44140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.5546875" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -966,7 +955,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1010,7 +999,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1051,7 +1040,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1072,7 +1061,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1110,7 +1099,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1148,7 +1137,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1177,7 +1166,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1200,7 +1189,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1229,7 +1218,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1261,7 +1250,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1296,7 +1285,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1322,7 +1311,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1357,7 +1346,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1380,7 +1369,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1415,7 +1404,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1438,10 +1427,13 @@
         <v>174</v>
       </c>
       <c r="I16" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.4">
+        <v>89</v>
+      </c>
+      <c r="K16">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1458,7 +1450,7 @@
         <v>91</v>
       </c>
       <c r="F17" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H17">
         <v>935</v>
@@ -1467,7 +1459,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1478,31 +1470,31 @@
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H18">
         <v>469</v>
       </c>
       <c r="I18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K18">
         <v>554</v>
       </c>
       <c r="L18" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="N18">
         <v>935</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1513,31 +1505,31 @@
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H19">
         <v>212</v>
       </c>
       <c r="I19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K19">
         <v>252</v>
       </c>
       <c r="L19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N19">
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1548,31 +1540,31 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H20">
         <v>382</v>
       </c>
       <c r="I20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K20">
         <v>636</v>
       </c>
       <c r="L20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N20">
         <v>282</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1583,37 +1575,37 @@
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H21">
         <v>389</v>
       </c>
       <c r="I21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K21">
         <v>224</v>
       </c>
       <c r="L21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N21">
         <v>470</v>
       </c>
       <c r="O21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q21">
         <v>315</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1624,25 +1616,25 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H22">
         <v>361</v>
       </c>
       <c r="I22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K22">
         <v>419</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1653,25 +1645,25 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H23" s="3">
         <v>591</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K23">
         <v>387</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1682,19 +1674,19 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H24">
         <v>377</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1705,25 +1697,25 @@
         <v>3</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H25">
         <v>561</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K25">
         <v>499</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -1734,31 +1726,31 @@
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H26">
         <v>760</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K26">
         <v>223</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N26">
         <v>215</v>
       </c>
     </row>
-    <row r="27" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1769,28 +1761,28 @@
         <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F27" s="3"/>
       <c r="I27" s="3"/>
       <c r="L27" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N27">
         <v>275</v>
       </c>
       <c r="O27" s="3"/>
       <c r="R27" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="T27">
         <v>450</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -1801,13 +1793,13 @@
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E28" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.4">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -1818,13 +1810,13 @@
         <v>7</v>
       </c>
       <c r="D29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E29" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.4">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -1835,13 +1827,13 @@
         <v>8</v>
       </c>
       <c r="D30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E30" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -1852,40 +1844,40 @@
         <v>9</v>
       </c>
       <c r="D31" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E31" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H31">
         <v>434</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K31">
         <v>274</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N31">
         <v>470</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q31">
         <v>764</v>
       </c>
       <c r="U31" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.4">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -1893,7 +1885,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -1904,19 +1896,19 @@
         <v>8</v>
       </c>
       <c r="D33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E33" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H33">
         <v>567</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>21</v>
       </c>
@@ -1924,782 +1916,782 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>21</v>
       </c>
@@ -2712,16 +2704,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
-    <col min="238" max="243" width="11.07421875" style="1" customWidth="1"/>
-    <col min="244" max="16384" width="11.07421875" style="1"/>
+    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
+    <col min="238" max="244" width="11.109375" style="1" customWidth="1"/>
+    <col min="245" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -3434,7 +3426,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -3443,13 +3435,13 @@
       </c>
       <c r="H2" s="2"/>
       <c r="V2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AF2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -3458,13 +3450,13 @@
       </c>
       <c r="H3" s="2"/>
       <c r="W3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AE3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -3473,10 +3465,10 @@
       </c>
       <c r="H4" s="2"/>
       <c r="Y4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -3485,13 +3477,13 @@
       </c>
       <c r="H5" s="2"/>
       <c r="Y5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AC5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -3500,19 +3492,19 @@
       </c>
       <c r="H6" s="2"/>
       <c r="AD6" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -3521,7 +3513,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -3530,13 +3522,13 @@
       </c>
       <c r="H9" s="2"/>
       <c r="AA9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AC9" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -3545,13 +3537,13 @@
       </c>
       <c r="H10" s="2"/>
       <c r="AA10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AE10" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -3560,10 +3552,10 @@
       </c>
       <c r="H11" s="2"/>
       <c r="AA11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -3572,7 +3564,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -3581,13 +3573,13 @@
       </c>
       <c r="H13" s="2"/>
       <c r="AB13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AE13" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -3596,7 +3588,7 @@
       </c>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -3605,7 +3597,7 @@
       </c>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -3614,7 +3606,7 @@
       </c>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -3623,733 +3615,733 @@
       </c>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B30" t="s">
+        <v>141</v>
+      </c>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>142</v>
+      </c>
+      <c r="B31" t="s">
+        <v>143</v>
+      </c>
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>140</v>
       </c>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A31" t="s">
-        <v>141</v>
-      </c>
-      <c r="B31" t="s">
-        <v>142</v>
-      </c>
-      <c r="H31" s="2"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A33" t="s">
-        <v>139</v>
-      </c>
       <c r="B33" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="230" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H230" s="2"/>
     </row>
   </sheetData>
@@ -4360,12 +4352,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>37</v>
       </c>
@@ -4385,10 +4377,10 @@
         <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J1">
         <v>45</v>
@@ -4412,10 +4404,10 @@
         <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="R1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -4436,10 +4428,10 @@
         <v>6</v>
       </c>
       <c r="Y1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Z1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AA1">
         <v>9</v>
@@ -4460,10 +4452,10 @@
         <v>14</v>
       </c>
       <c r="AG1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AH1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AI1">
         <v>17</v>
@@ -4493,88 +4485,88 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -4585,17 +4577,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>37</v>
       </c>
@@ -4603,7 +4595,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>37</v>
       </c>
@@ -4611,7 +4603,7 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>37</v>
       </c>
@@ -4619,7 +4611,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>37</v>
       </c>
@@ -4627,7 +4619,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>37</v>
       </c>
@@ -4635,7 +4627,7 @@
         <v>46276</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>37</v>
       </c>
@@ -4643,7 +4635,7 @@
         <v>46277</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>37</v>
       </c>
@@ -4651,7 +4643,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>38</v>
       </c>
@@ -4659,7 +4651,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>38</v>
       </c>
@@ -4667,7 +4659,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>38</v>
       </c>
@@ -4675,7 +4667,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>38</v>
       </c>
@@ -4683,7 +4675,7 @@
         <v>46282</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>38</v>
       </c>
@@ -4691,7 +4683,7 @@
         <v>46283</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>38</v>
       </c>
@@ -4699,7 +4691,7 @@
         <v>46284</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 24-09-2026 14:02:58.85
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" state="visible" r:id="rId1"/>
@@ -1349,7 +1349,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="21" s="1">
+    <row r="21">
       <c r="A21" t="inlineStr">
         <is>
           <t>T</t>
@@ -1396,7 +1396,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="22" s="1">
+    <row r="22">
       <c r="A22" t="inlineStr">
         <is>
           <t>T</t>
@@ -2981,8 +2981,8 @@
     <col width="11.109375" customWidth="1" style="1" min="1" max="1"/>
     <col width="60" customWidth="1" style="1" min="2" max="2"/>
     <col width="2.6640625" customWidth="1" style="1" min="3" max="237"/>
-    <col width="11.109375" customWidth="1" style="1" min="238" max="245"/>
-    <col width="11.109375" customWidth="1" style="1" min="246" max="16384"/>
+    <col width="11.109375" customWidth="1" style="1" min="238" max="246"/>
+    <col width="11.109375" customWidth="1" style="1" min="247" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="59.1" customHeight="1" s="1">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Discuter la coplanarité de vecteur (avec coord)</t>
+          <t>Calculer des coordonnées de points</t>
         </is>
       </c>
       <c r="H18" s="2" t="n"/>
@@ -4086,10 +4086,15 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Construire une section de cube</t>
+          <t>Discuter la colinéarité de vecteur (avec coord)</t>
         </is>
       </c>
       <c r="H19" s="2" t="n"/>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4099,10 +4104,15 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Construire une section de cube</t>
+          <t>Discuter la coplanarité de vecteur (avec coord)</t>
         </is>
       </c>
       <c r="H20" s="2" t="n"/>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4112,7 +4122,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Etudier une suite à l'aide d'une fonction</t>
+          <t>Construire une section de cube</t>
         </is>
       </c>
       <c r="H21" s="2" t="n"/>
@@ -4125,7 +4135,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Représenter graphiquement une suite défini par une fonction</t>
+          <t>Construire une section de cube</t>
         </is>
       </c>
       <c r="H22" s="2" t="n"/>
@@ -4138,7 +4148,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
+          <t>Etudier une suite à l'aide d'une fonction support</t>
         </is>
       </c>
       <c r="H23" s="2" t="n"/>
@@ -4151,7 +4161,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Additionner des limites</t>
+          <t>Représenter graphiquement une suite défini par une fonction</t>
         </is>
       </c>
       <c r="H24" s="2" t="n"/>
@@ -4164,7 +4174,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Produit et Quotient de limite</t>
+          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
         </is>
       </c>
       <c r="H25" s="2" t="n"/>
@@ -4177,7 +4187,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Lever une indétermination en factorisant</t>
+          <t>Additionner des limites</t>
         </is>
       </c>
       <c r="H26" s="2" t="n"/>
@@ -4190,7 +4200,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Lever une indétermination avec des racines carrés</t>
+          <t>Produit et Quotient de limite</t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>
@@ -4203,7 +4213,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Utiliser le théorème de comparaison</t>
+          <t>Lever une indétermination en factorisant</t>
         </is>
       </c>
       <c r="H28" s="2" t="n"/>
@@ -4216,7 +4226,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
+          <t>Lever une indétermination avec des racines carrés</t>
         </is>
       </c>
       <c r="H29" s="2" t="n"/>
@@ -4229,7 +4239,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Justifier la convergence d'une suite</t>
+          <t>Utiliser le théorème de comparaison</t>
         </is>
       </c>
       <c r="H30" s="2" t="n"/>
@@ -4242,7 +4252,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Limite d'une suite géométrique</t>
+          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
         </is>
       </c>
       <c r="H31" s="2" t="n"/>
@@ -4268,7 +4278,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>a recaser</t>
+          <t>Limite d'une suite géométrique</t>
         </is>
       </c>
       <c r="H33" s="2" t="n"/>

</xml_diff>

<commit_message>
Mise a jour du 28-09-2026 16:35:56.20
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8170649E-BF6A-40E2-B226-EB8A98C57A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA962F8D-0009-4A84-B22A-70A3ACDC68BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="176">
   <si>
     <t>Préfixe</t>
   </si>
@@ -3655,6 +3655,9 @@
       <c r="AI13" t="s">
         <v>157</v>
       </c>
+      <c r="AN13" s="1" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -3694,8 +3697,11 @@
       <c r="AH16" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="AN16" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="17" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -3707,7 +3713,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -3718,8 +3724,11 @@
       <c r="AJ18" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="AO18" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -3730,8 +3739,11 @@
       <c r="AK19" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="AO19" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="20" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -3742,8 +3754,11 @@
       <c r="AK20" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="AO20" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="21" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>107</v>
       </c>
@@ -3751,8 +3766,11 @@
         <v>108</v>
       </c>
       <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="AM21" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="22" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>112</v>
       </c>
@@ -3760,8 +3778,11 @@
         <v>108</v>
       </c>
       <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="AM22" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="23" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>115</v>
       </c>
@@ -3770,7 +3791,7 @@
       </c>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>120</v>
       </c>
@@ -3779,7 +3800,7 @@
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>123</v>
       </c>
@@ -3788,7 +3809,7 @@
       </c>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>127</v>
       </c>
@@ -3797,7 +3818,7 @@
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>130</v>
       </c>
@@ -3806,7 +3827,7 @@
       </c>
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>134</v>
       </c>
@@ -3815,7 +3836,7 @@
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>139</v>
       </c>
@@ -3824,7 +3845,7 @@
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -3833,7 +3854,7 @@
       </c>
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>145</v>
       </c>
@@ -3842,7 +3863,7 @@
       </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>147</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 29-09-2026 15:49:35,01
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA962F8D-0009-4A84-B22A-70A3ACDC68BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F359EC77-7CA7-4008-B83B-08CA9E612523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="176">
   <si>
     <t>Préfixe</t>
   </si>
@@ -882,27 +882,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U192"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="3.88671875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="3.88671875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="2.44140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.84375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.69140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.53515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.23046875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="3.84375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.23046875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.84375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.84375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="3.84375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="2.4609375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.53515625" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -967,7 +967,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1410,19 +1410,13 @@
         <v>84</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H15">
-        <v>935</v>
-      </c>
-      <c r="I15" t="s">
-        <v>86</v>
-      </c>
-      <c r="K15">
         <v>289</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1457,7 +1451,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1480,7 +1474,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1509,7 +1503,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1538,7 +1532,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1573,7 +1567,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1608,7 +1602,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1637,7 +1631,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" ht="28.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1672,7 +1666,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" ht="28.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1695,7 +1689,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1724,7 +1718,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -1747,7 +1741,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1776,7 +1770,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -1811,7 +1805,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -1843,7 +1837,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -1860,7 +1854,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -1877,7 +1871,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" ht="28.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -1900,7 +1894,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -1944,7 +1938,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>21</v>
       </c>
@@ -1952,792 +1946,792 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A122" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A123" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A128" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A130" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A131" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A135" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A136" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A137" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A138" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A139" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A140" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A141" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A142" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A143" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A144" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A145" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A146" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A147" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A148" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A149" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A150" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A151" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A152" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A153" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A154" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A155" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A156" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A157" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A158" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A159" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A160" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A161" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A162" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A163" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A164" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A165" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A166" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A167" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A168" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A169" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A170" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A171" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A172" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A173" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A174" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A175" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A176" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A177" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A178" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A179" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A180" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A181" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A182" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A183" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A184" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A185" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A186" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A187" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A188" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A189" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A190" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A191" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A192" t="s">
         <v>21</v>
       </c>
@@ -2750,16 +2744,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
-    <col min="238" max="247" width="11.109375" style="1" customWidth="1"/>
-    <col min="248" max="16384" width="11.109375" style="1"/>
+    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
+    <col min="238" max="247" width="11.07421875" style="1" customWidth="1"/>
+    <col min="248" max="16384" width="11.07421875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -3472,7 +3466,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -3490,7 +3484,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -3508,7 +3502,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -3526,7 +3520,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -3545,7 +3539,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -3560,7 +3554,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -3569,7 +3563,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -3578,7 +3572,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -3596,7 +3590,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -3614,7 +3608,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -3629,7 +3623,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>71</v>
       </c>
@@ -3638,7 +3632,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -3659,7 +3653,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>79</v>
       </c>
@@ -3674,7 +3668,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -3685,8 +3679,11 @@
       <c r="AH15" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
+      <c r="AN15" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -3701,7 +3698,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -3712,8 +3709,11 @@
       <c r="AI17" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="18" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="AN17" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -3728,7 +3728,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -3758,7 +3758,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="21" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>107</v>
       </c>
@@ -3770,7 +3770,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="22" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>112</v>
       </c>
@@ -3782,7 +3782,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="23" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>115</v>
       </c>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>120</v>
       </c>
@@ -3800,7 +3800,7 @@
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>123</v>
       </c>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>127</v>
       </c>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>130</v>
       </c>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>134</v>
       </c>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>139</v>
       </c>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>145</v>
       </c>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>147</v>
       </c>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>143</v>
       </c>
@@ -3881,595 +3881,595 @@
       </c>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H230" s="2"/>
     </row>
   </sheetData>
@@ -4480,12 +4480,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
       <c r="B1">
         <v>37</v>
       </c>
@@ -4613,7 +4613,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>159</v>
       </c>
@@ -4627,72 +4627,72 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>173</v>
       </c>
@@ -4705,9 +4705,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>174</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>37</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>37</v>
       </c>
@@ -4731,7 +4731,7 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>37</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>37</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>37</v>
       </c>
@@ -4755,7 +4755,7 @@
         <v>46276</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>37</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>46277</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>37</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>38</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>38</v>
       </c>
@@ -4787,7 +4787,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>38</v>
       </c>
@@ -4795,7 +4795,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>38</v>
       </c>
@@ -4803,7 +4803,7 @@
         <v>46282</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>38</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>46283</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>38</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>46284</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 05-10-2026 16:55:53.81
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F359EC77-7CA7-4008-B83B-08CA9E612523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{659C9DE0-6525-4489-B18C-16717D8106D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="173">
   <si>
     <t>Préfixe</t>
   </si>
@@ -447,18 +447,6 @@
     <t>jCFejEo2oQY</t>
   </si>
   <si>
-    <t>T.SF3.7</t>
-  </si>
-  <si>
-    <t>Lever une indétermination avec des racines carrés</t>
-  </si>
-  <si>
-    <t>JbDvz3iobMk</t>
-  </si>
-  <si>
-    <t>HNxF6K5mvvk</t>
-  </si>
-  <si>
     <t>T.SF3.8</t>
   </si>
   <si>
@@ -556,6 +544,9 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Construire une section d'un tétraèdre</t>
   </si>
 </sst>
 </file>
@@ -591,7 +582,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -601,6 +592,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -881,28 +873,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U192"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:U191"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.84375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.69140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.53515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.23046875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="3.84375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.23046875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.84375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.84375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="3.84375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="2.4609375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.53515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="3.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="3.88671875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="2.44140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.5546875" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -967,7 +959,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1011,7 +1003,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1052,7 +1044,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1073,7 +1065,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1111,7 +1103,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1149,7 +1141,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1178,7 +1170,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1207,7 +1199,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1239,7 +1231,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1265,7 +1257,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1303,7 +1295,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1329,7 +1321,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1364,7 +1356,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1393,7 +1385,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1416,7 +1408,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1451,7 +1443,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1474,7 +1466,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1503,7 +1495,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1532,7 +1524,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1567,7 +1559,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1601,8 +1593,14 @@
       <c r="N21">
         <v>470</v>
       </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="O21" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q21" s="1">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1616,7 +1614,7 @@
         <v>112</v>
       </c>
       <c r="E22" t="s">
-        <v>108</v>
+        <v>172</v>
       </c>
       <c r="F22" t="s">
         <v>113</v>
@@ -1631,7 +1629,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="28.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1666,7 +1664,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="28.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1689,7 +1687,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1718,7 +1716,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -1741,7 +1739,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1770,15 +1768,15 @@
         <v>499</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>21</v>
       </c>
       <c r="B28">
         <v>3</v>
       </c>
-      <c r="C28">
-        <v>6</v>
+      <c r="C28" s="5">
+        <v>46209</v>
       </c>
       <c r="D28" t="s">
         <v>134</v>
@@ -1805,7 +1803,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -1813,7 +1811,7 @@
         <v>3</v>
       </c>
       <c r="C29">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D29" t="s">
         <v>139</v>
@@ -1821,23 +1819,8 @@
       <c r="E29" t="s">
         <v>140</v>
       </c>
-      <c r="F29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="L29" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="N29">
-        <v>275</v>
-      </c>
-      <c r="O29" s="3"/>
-      <c r="R29" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="T29">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -1845,16 +1828,16 @@
         <v>3</v>
       </c>
       <c r="C30">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D30" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E30" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -1862,16 +1845,22 @@
         <v>3</v>
       </c>
       <c r="C31">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D31" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31" t="s">
+        <v>144</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E31" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" ht="28.85" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="H31">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -1879,860 +1868,837 @@
         <v>3</v>
       </c>
       <c r="C32">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D32" t="s">
+        <v>146</v>
+      </c>
+      <c r="E32" t="s">
         <v>147</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="H32">
+        <v>434</v>
+      </c>
+      <c r="I32" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="H32">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K32">
+        <v>274</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="N32">
+        <v>470</v>
+      </c>
+      <c r="O32" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q32">
+        <v>764</v>
+      </c>
+      <c r="U32" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>21</v>
       </c>
       <c r="B33">
-        <v>3</v>
-      </c>
-      <c r="C33">
-        <v>11</v>
-      </c>
-      <c r="D33" t="s">
-        <v>150</v>
-      </c>
-      <c r="E33" t="s">
-        <v>151</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="H33">
-        <v>434</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="K33">
-        <v>274</v>
-      </c>
-      <c r="L33" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="N33">
-        <v>470</v>
-      </c>
-      <c r="O33" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q33">
-        <v>764</v>
-      </c>
-      <c r="U33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>21</v>
       </c>
-      <c r="B34">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A192" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2743,17 +2709,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:IC229"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
-    <col min="238" max="247" width="11.07421875" style="1" customWidth="1"/>
-    <col min="248" max="16384" width="11.07421875" style="1"/>
+    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
+    <col min="238" max="247" width="11.109375" style="1" customWidth="1"/>
+    <col min="248" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -3466,7 +3432,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -3475,16 +3441,16 @@
       </c>
       <c r="H2" s="2"/>
       <c r="V2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AF2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AL2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -3493,16 +3459,19 @@
       </c>
       <c r="H3" s="2"/>
       <c r="W3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AE3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AL3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+      <c r="AT3" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -3511,16 +3480,16 @@
       </c>
       <c r="H4" s="2"/>
       <c r="Y4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AJ4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AL4" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -3529,17 +3498,20 @@
       </c>
       <c r="H5" s="2"/>
       <c r="Y5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AC5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AK5"/>
       <c r="AL5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+      <c r="AS5" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -3548,13 +3520,13 @@
       </c>
       <c r="H6" s="2"/>
       <c r="AD6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AL6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -3563,7 +3535,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -3572,7 +3544,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -3581,16 +3553,16 @@
       </c>
       <c r="H9" s="2"/>
       <c r="AA9" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AC9" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AI9" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -3599,16 +3571,16 @@
       </c>
       <c r="H10" s="2"/>
       <c r="AA10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AE10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AJ10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -3617,13 +3589,13 @@
       </c>
       <c r="H11" s="2"/>
       <c r="AA11" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AJ11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>71</v>
       </c>
@@ -3632,7 +3604,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -3641,19 +3613,19 @@
       </c>
       <c r="H13" s="2"/>
       <c r="AB13" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AE13" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AI13" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AN13" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>79</v>
       </c>
@@ -3662,13 +3634,13 @@
       </c>
       <c r="H14" s="2"/>
       <c r="AH14" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AM14" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -3677,13 +3649,13 @@
       </c>
       <c r="H15" s="2"/>
       <c r="AH15" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AN15" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -3692,13 +3664,13 @@
       </c>
       <c r="H16" s="2"/>
       <c r="AH16" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AN16" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="17" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -3707,13 +3679,13 @@
       </c>
       <c r="H17" s="2"/>
       <c r="AI17" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AN17" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="18" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -3722,13 +3694,13 @@
       </c>
       <c r="H18" s="2"/>
       <c r="AJ18" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AO18" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="19" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -3737,13 +3709,13 @@
       </c>
       <c r="H19" s="2"/>
       <c r="AK19" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AO19" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="20" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -3752,13 +3724,13 @@
       </c>
       <c r="H20" s="2"/>
       <c r="AK20" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AO20" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>107</v>
       </c>
@@ -3767,10 +3739,10 @@
       </c>
       <c r="H21" s="2"/>
       <c r="AM21" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="22" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="22" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>112</v>
       </c>
@@ -3779,10 +3751,10 @@
       </c>
       <c r="H22" s="2"/>
       <c r="AM22" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="23" spans="1:41" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>115</v>
       </c>
@@ -3790,8 +3762,11 @@
         <v>116</v>
       </c>
       <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AR23" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>120</v>
       </c>
@@ -3799,8 +3774,11 @@
         <v>121</v>
       </c>
       <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AR24" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>123</v>
       </c>
@@ -3808,8 +3786,11 @@
         <v>124</v>
       </c>
       <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AS25" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>127</v>
       </c>
@@ -3818,7 +3799,7 @@
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>130</v>
       </c>
@@ -3827,7 +3808,7 @@
       </c>
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>134</v>
       </c>
@@ -3836,7 +3817,7 @@
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>139</v>
       </c>
@@ -3845,632 +3826,623 @@
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>141</v>
+      </c>
+      <c r="B30" t="s">
+        <v>142</v>
+      </c>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="1:45" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>143</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>144</v>
       </c>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:41" x14ac:dyDescent="0.4">
-      <c r="A31" t="s">
-        <v>145</v>
-      </c>
-      <c r="B31" t="s">
-        <v>146</v>
-      </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>139</v>
+      </c>
+      <c r="B32" t="s">
         <v>147</v>
       </c>
-      <c r="B32" t="s">
-        <v>148</v>
-      </c>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A33" t="s">
-        <v>143</v>
-      </c>
-      <c r="B33" t="s">
-        <v>151</v>
-      </c>
+    <row r="33" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="36" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="37" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="39" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="40" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="42" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="43" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="45" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="46" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="48" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H229" s="2"/>
-    </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
-      <c r="H230" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4480,12 +4452,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>37</v>
       </c>
@@ -4505,10 +4477,10 @@
         <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="J1">
         <v>45</v>
@@ -4532,10 +4504,10 @@
         <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="R1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -4556,10 +4528,10 @@
         <v>6</v>
       </c>
       <c r="Y1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="Z1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="AA1">
         <v>9</v>
@@ -4580,10 +4552,10 @@
         <v>14</v>
       </c>
       <c r="AG1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="AH1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="AI1">
         <v>17</v>
@@ -4613,88 +4585,88 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>159</v>
       </c>
-      <c r="B2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A15" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
-      <c r="A16" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -4705,17 +4677,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>37</v>
       </c>
@@ -4723,7 +4695,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>37</v>
       </c>
@@ -4731,7 +4703,7 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>37</v>
       </c>
@@ -4739,7 +4711,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>37</v>
       </c>
@@ -4747,7 +4719,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>37</v>
       </c>
@@ -4755,7 +4727,7 @@
         <v>46276</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>37</v>
       </c>
@@ -4763,7 +4735,7 @@
         <v>46277</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>37</v>
       </c>
@@ -4771,7 +4743,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>38</v>
       </c>
@@ -4779,7 +4751,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>38</v>
       </c>
@@ -4787,7 +4759,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>38</v>
       </c>
@@ -4795,7 +4767,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>38</v>
       </c>
@@ -4803,7 +4775,7 @@
         <v>46282</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>38</v>
       </c>
@@ -4811,7 +4783,7 @@
         <v>46283</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>38</v>
       </c>
@@ -4819,7 +4791,7 @@
         <v>46284</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 09-10-2026 12:48:22,97
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED30A50-2112-47FA-BC96-EE8D6CAC41EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4310A49F-7896-43F8-8186-3E23CCDE540E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="176">
   <si>
     <t>Préfixe</t>
   </si>
@@ -3699,7 +3699,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -3729,7 +3729,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>108</v>
       </c>
@@ -3771,7 +3771,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>113</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>117</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>124</v>
       </c>
@@ -3809,8 +3809,11 @@
       <c r="AR24" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.4">
+      <c r="AV24" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>127</v>
       </c>
@@ -3821,8 +3824,11 @@
       <c r="AS25" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.4">
+      <c r="AV25" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="26" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>131</v>
       </c>
@@ -3830,8 +3836,11 @@
         <v>132</v>
       </c>
       <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.4">
+      <c r="AV26" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="27" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>134</v>
       </c>
@@ -3839,8 +3848,11 @@
         <v>135</v>
       </c>
       <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.4">
+      <c r="AV27" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="28" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>138</v>
       </c>
@@ -3849,7 +3861,7 @@
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>143</v>
       </c>
@@ -3858,7 +3870,7 @@
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>145</v>
       </c>
@@ -3867,7 +3879,7 @@
       </c>
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>147</v>
       </c>
@@ -3876,7 +3888,7 @@
       </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:48" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>150</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 12-10-2026 11:16:20,22
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4310A49F-7896-43F8-8186-3E23CCDE540E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E8788D-FDFB-4BCB-B2AF-00460F520A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="176">
   <si>
     <t>Préfixe</t>
   </si>
@@ -3699,7 +3699,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="18" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -3729,7 +3729,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="21" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>108</v>
       </c>
@@ -3771,7 +3771,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="22" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>113</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="23" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>117</v>
       </c>
@@ -3797,8 +3797,11 @@
       <c r="AU23" s="1" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="24" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AY23" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="24" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>124</v>
       </c>
@@ -3812,8 +3815,11 @@
       <c r="AV24" s="1" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="25" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AY24" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>127</v>
       </c>
@@ -3828,7 +3834,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>131</v>
       </c>
@@ -3840,7 +3846,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="27" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>134</v>
       </c>
@@ -3852,7 +3858,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="28" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>138</v>
       </c>
@@ -3861,7 +3867,7 @@
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>143</v>
       </c>
@@ -3870,7 +3876,7 @@
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>145</v>
       </c>
@@ -3879,7 +3885,7 @@
       </c>
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>147</v>
       </c>
@@ -3888,7 +3894,7 @@
       </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:51" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>150</v>
       </c>

</xml_diff>